<commit_message>
auto(MT): 3h refresh 2026-05-17T16:57Z
</commit_message>
<xml_diff>
--- a/daily_report_mt_2026-05-17.xlsx
+++ b/daily_report_mt_2026-05-17.xlsx
@@ -611,7 +611,6 @@
           <t>PL</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>Ray Abela</t>
@@ -733,7 +732,6 @@
           <t>PN</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>Michael Piccinino</t>
@@ -855,7 +853,6 @@
           <t>PN</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>Michael Piccinino</t>
@@ -886,7 +883,6 @@
           <t>2026-05-14</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>0–99</t>
@@ -925,7 +921,7 @@
   <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -1013,10 +1009,75 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>No re-advertisers detected.</t>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Politician</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Page Name</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Page ID</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>New Ad ID</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>View Ad</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>New Ad Start</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>New Ad Stop</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>First Removal Detected</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>Total Ads Removed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto(MT): 3h refresh 2026-05-17T21:02Z
</commit_message>
<xml_diff>
--- a/daily_report_mt_2026-05-17.xlsx
+++ b/daily_report_mt_2026-05-17.xlsx
@@ -918,7 +918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1076,6 +1076,78 @@
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>Total Ads Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Politician</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Page Name</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Page ID</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>New Ad ID</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>View Ad</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>New Ad Start</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>New Ad Stop</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>First Removal Detected</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>Total Ads Removed</t>
         </is>

</xml_diff>

<commit_message>
auto(MT): 3h refresh 2026-05-17T21:15Z
</commit_message>
<xml_diff>
--- a/daily_report_mt_2026-05-17.xlsx
+++ b/daily_report_mt_2026-05-17.xlsx
@@ -918,7 +918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1148,6 +1148,78 @@
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>Total Ads Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Politician</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Page Name</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Page ID</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>New Ad ID</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>View Ad</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>New Ad Start</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>New Ad Stop</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>First Removal Detected</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Total Ads Removed</t>
         </is>

</xml_diff>

<commit_message>
auto(MT): 3h refresh 2026-05-17T21:25Z
</commit_message>
<xml_diff>
--- a/daily_report_mt_2026-05-17.xlsx
+++ b/daily_report_mt_2026-05-17.xlsx
@@ -918,7 +918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1220,6 +1220,78 @@
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>Total Ads Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Politician</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Page Name</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Page ID</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>New Ad ID</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>View Ad</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>New Ad Start</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>New Ad Stop</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="M5" s="5" t="inlineStr">
+        <is>
+          <t>First Removal Detected</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Total Ads Removed</t>
         </is>

</xml_diff>

<commit_message>
auto(MT): 3h refresh 2026-05-17T22:40Z
</commit_message>
<xml_diff>
--- a/daily_report_mt_2026-05-17.xlsx
+++ b/daily_report_mt_2026-05-17.xlsx
@@ -918,7 +918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1292,6 +1292,78 @@
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>Total Ads Removed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Politician</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Page Name</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Page ID</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>New Ad ID</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>View Ad</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>New Ad Start</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>New Ad Stop</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>First Removal Detected</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>Total Ads Removed</t>
         </is>

</xml_diff>